<commit_message>
Stream mapped inputs and all-read reports; accelerate Shiny with live validation
</commit_message>
<xml_diff>
--- a/example/reference_results/2_quality_filtered_reads/quality_and_read_length_summary.xlsx
+++ b/example/reference_results/2_quality_filtered_reads/quality_and_read_length_summary.xlsx
@@ -159,11 +159,59 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Maximum deterministic observations retained per sample for plots and quantiles.</t>
+          <t xml:space="preserve">Maximum sample facets per distribution PDF page (six).</t>
         </r>
       </text>
     </comment>
     <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Width of the all-read length histogram bins in base pairs.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Width of the all-read QV histogram bins in QV units.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="O1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Inclusive minimum read length in the count annotated in each read-length facet.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="P1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Inclusive maximum read length in the count annotated in each read-length facet.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Q1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -289,7 +337,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Fifth percentile read length estimated from the bounded plotting sample.</t>
+          <t xml:space="preserve">Fifth percentile read length calculated exactly from all input read-length frequencies.</t>
         </r>
       </text>
     </comment>
@@ -301,7 +349,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Twenty-fifth percentile read length estimated from the bounded plotting sample.</t>
+          <t xml:space="preserve">Twenty-fifth percentile read length calculated exactly from all input read-length frequencies.</t>
         </r>
       </text>
     </comment>
@@ -313,7 +361,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Median read length estimated from the bounded plotting sample.</t>
+          <t xml:space="preserve">Median read length calculated exactly from all input read-length frequencies.</t>
         </r>
       </text>
     </comment>
@@ -325,7 +373,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Seventy-fifth percentile read length estimated from the bounded plotting sample.</t>
+          <t xml:space="preserve">Seventy-fifth percentile read length calculated exactly from all input read-length frequencies.</t>
         </r>
       </text>
     </comment>
@@ -337,7 +385,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Ninety-fifth percentile read length estimated from the bounded plotting sample.</t>
+          <t xml:space="preserve">Ninety-fifth percentile read length calculated exactly from all input read-length frequencies.</t>
         </r>
       </text>
     </comment>
@@ -349,11 +397,23 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
+          <t xml:space="preserve">Input reads between AnnotationLengthMinimum (1800) and AnnotationLengthMaximum (2000), inclusive.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="O1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
           <t xml:space="preserve">Reads between the configured expected minimum and maximum lengths, inclusive.</t>
         </r>
       </text>
     </comment>
-    <comment ref="O1" authorId="0" shapeId="0">
+    <comment ref="P1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -365,7 +425,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P1" authorId="0" shapeId="0">
+    <comment ref="Q1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -377,7 +437,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q1" authorId="0" shapeId="0">
+    <comment ref="R1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -389,7 +449,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="R1" authorId="0" shapeId="0">
+    <comment ref="S1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -401,7 +461,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S1" authorId="0" shapeId="0">
+    <comment ref="T1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -413,7 +473,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="T1" authorId="0" shapeId="0">
+    <comment ref="U1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -425,7 +485,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="U1" authorId="0" shapeId="0">
+    <comment ref="V1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -437,7 +497,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="V1" authorId="0" shapeId="0">
+    <comment ref="W1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -449,7 +509,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="W1" authorId="0" shapeId="0">
+    <comment ref="X1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -461,7 +521,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="X1" authorId="0" shapeId="0">
+    <comment ref="Y1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -473,7 +533,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Y1" authorId="0" shapeId="0">
+    <comment ref="Z1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -485,18 +545,6 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <name val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Reads retained in the bounded deterministic plotting and quantile sample.</t>
-        </r>
-      </text>
-    </comment>
     <comment ref="AA1" authorId="0" shapeId="0">
       <text>
         <r>
@@ -505,11 +553,23 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
+          <t xml:space="preserve">All input reads counted in the distribution histograms; equals TotalReads.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AB1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
           <t xml:space="preserve">PASS when at least one read passes the configured QV filter; otherwise REVIEW.</t>
         </r>
       </text>
     </comment>
-    <comment ref="AB1" authorId="0" shapeId="0">
+    <comment ref="AC1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -521,7 +581,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AC1" authorId="0" shapeId="0">
+    <comment ref="AD1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -584,7 +644,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="99">
   <si>
     <t xml:space="preserve">PoolNumber</t>
   </si>
@@ -619,7 +679,19 @@
     <t xml:space="preserve">StreamYieldSize</t>
   </si>
   <si>
-    <t xml:space="preserve">MaximumPlotReadsPerSample</t>
+    <t xml:space="preserve">SamplesPerPlotPage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LengthHistogramBinWidth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QVHistogramBinWidth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AnnotationLengthMinimum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AnnotationLengthMaximum</t>
   </si>
   <si>
     <t xml:space="preserve">OverallQCStatus</t>
@@ -667,6 +739,9 @@
     <t xml:space="preserve">LengthP95</t>
   </si>
   <si>
+    <t xml:space="preserve">ReadsInAnnotationRange</t>
+  </si>
+  <si>
     <t xml:space="preserve">ReadsInExpectedLengthRange</t>
   </si>
   <si>
@@ -748,7 +823,19 @@
     <t xml:space="preserve">Maximum FASTQ records read into memory per streaming yield.</t>
   </si>
   <si>
-    <t xml:space="preserve">Maximum deterministic observations retained per sample for plots and quantiles.</t>
+    <t xml:space="preserve">Maximum sample facets per distribution PDF page (six).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Width of the all-read length histogram bins in base pairs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Width of the all-read QV histogram bins in QV units.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inclusive minimum read length in the count annotated in each read-length facet.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inclusive maximum read length in the count annotated in each read-length facet.</t>
   </si>
   <si>
     <t xml:space="preserve">PASS when both QualityStatus and LengthStatus pass; otherwise REVIEW.</t>
@@ -769,19 +856,22 @@
     <t xml:space="preserve">Longest read length in base pairs.</t>
   </si>
   <si>
-    <t xml:space="preserve">Fifth percentile read length estimated from the bounded plotting sample.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Twenty-fifth percentile read length estimated from the bounded plotting sample.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Median read length estimated from the bounded plotting sample.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Seventy-fifth percentile read length estimated from the bounded plotting sample.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ninety-fifth percentile read length estimated from the bounded plotting sample.</t>
+    <t xml:space="preserve">Fifth percentile read length calculated exactly from all input read-length frequencies.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Twenty-fifth percentile read length calculated exactly from all input read-length frequencies.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Median read length calculated exactly from all input read-length frequencies.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seventy-fifth percentile read length calculated exactly from all input read-length frequencies.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ninety-fifth percentile read length calculated exactly from all input read-length frequencies.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Input reads between AnnotationLengthMinimum (1800) and AnnotationLengthMaximum (2000), inclusive.</t>
   </si>
   <si>
     <t xml:space="preserve">Reads between the configured expected minimum and maximum lengths, inclusive.</t>
@@ -811,7 +901,7 @@
     <t xml:space="preserve">Total bases among reads retained by the QV filter.</t>
   </si>
   <si>
-    <t xml:space="preserve">Reads retained in the bounded deterministic plotting and quantile sample.</t>
+    <t xml:space="preserve">All input reads counted in the distribution histograms; equals TotalReads.</t>
   </si>
   <si>
     <t xml:space="preserve">PASS when at least one read passes the configured QV filter; otherwise REVIEW.</t>
@@ -907,9 +997,9 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:M5" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:M5"/>
-  <tableColumns count="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:Q5" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:Q5"/>
+  <tableColumns count="17">
     <tableColumn id="1" name="PoolNumber"/>
     <tableColumn id="2" name="SampleID"/>
     <tableColumn id="3" name="TotalReads"/>
@@ -921,17 +1011,21 @@
     <tableColumn id="9" name="ExpectedLengthMaximum"/>
     <tableColumn id="10" name="ReadQVCutoff"/>
     <tableColumn id="11" name="StreamYieldSize"/>
-    <tableColumn id="12" name="MaximumPlotReadsPerSample"/>
-    <tableColumn id="13" name="OverallQCStatus"/>
+    <tableColumn id="12" name="SamplesPerPlotPage"/>
+    <tableColumn id="13" name="LengthHistogramBinWidth"/>
+    <tableColumn id="14" name="QVHistogramBinWidth"/>
+    <tableColumn id="15" name="AnnotationLengthMinimum"/>
+    <tableColumn id="16" name="AnnotationLengthMaximum"/>
+    <tableColumn id="17" name="OverallQCStatus"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Table4" displayName="Table4" ref="A1:AC5" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:AC5"/>
-  <tableColumns count="29">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Table4" displayName="Table4" ref="A1:AD5" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:AD5"/>
+  <tableColumns count="30">
     <tableColumn id="1" name="PoolNumber"/>
     <tableColumn id="2" name="SampleID"/>
     <tableColumn id="3" name="TotalReads"/>
@@ -945,30 +1039,31 @@
     <tableColumn id="11" name="MedianLength"/>
     <tableColumn id="12" name="LengthP75"/>
     <tableColumn id="13" name="LengthP95"/>
-    <tableColumn id="14" name="ReadsInExpectedLengthRange"/>
-    <tableColumn id="15" name="PercentInExpectedLengthRange"/>
-    <tableColumn id="16" name="MeanGCPercent"/>
-    <tableColumn id="17" name="MinimumReadQV"/>
-    <tableColumn id="18" name="MeanReadQV"/>
-    <tableColumn id="19" name="ReadQVSD"/>
-    <tableColumn id="20" name="MaximumReadQV"/>
-    <tableColumn id="21" name="QVCutoff"/>
-    <tableColumn id="22" name="PassingReads"/>
-    <tableColumn id="23" name="FilteredReads"/>
-    <tableColumn id="24" name="PercentPassingQV"/>
-    <tableColumn id="25" name="PassingBases"/>
-    <tableColumn id="26" name="PlotReads"/>
-    <tableColumn id="27" name="QualityStatus"/>
-    <tableColumn id="28" name="LengthStatus"/>
-    <tableColumn id="29" name="OverallQCStatus"/>
+    <tableColumn id="14" name="ReadsInAnnotationRange"/>
+    <tableColumn id="15" name="ReadsInExpectedLengthRange"/>
+    <tableColumn id="16" name="PercentInExpectedLengthRange"/>
+    <tableColumn id="17" name="MeanGCPercent"/>
+    <tableColumn id="18" name="MinimumReadQV"/>
+    <tableColumn id="19" name="MeanReadQV"/>
+    <tableColumn id="20" name="ReadQVSD"/>
+    <tableColumn id="21" name="MaximumReadQV"/>
+    <tableColumn id="22" name="QVCutoff"/>
+    <tableColumn id="23" name="PassingReads"/>
+    <tableColumn id="24" name="FilteredReads"/>
+    <tableColumn id="25" name="PercentPassingQV"/>
+    <tableColumn id="26" name="PassingBases"/>
+    <tableColumn id="27" name="PlotReads"/>
+    <tableColumn id="28" name="QualityStatus"/>
+    <tableColumn id="29" name="LengthStatus"/>
+    <tableColumn id="30" name="OverallQCStatus"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Table5" displayName="Table5" ref="A1:C49" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:C49"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Table5" displayName="Table5" ref="A1:C54" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:C54"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Sheet"/>
     <tableColumn id="2" name="Column"/>
@@ -1274,8 +1369,12 @@
     <col min="9" max="9" width="21.71" hidden="0" customWidth="1"/>
     <col min="10" max="10" width="12.71" hidden="0" customWidth="1"/>
     <col min="11" max="11" width="15.71" hidden="0" customWidth="1"/>
-    <col min="12" max="12" width="25.71" hidden="0" customWidth="1"/>
-    <col min="13" max="13" width="15.71" hidden="0" customWidth="1"/>
+    <col min="12" max="12" width="18.71" hidden="0" customWidth="1"/>
+    <col min="13" max="13" width="23.71" hidden="0" customWidth="1"/>
+    <col min="14" max="14" width="19.71" hidden="0" customWidth="1"/>
+    <col min="15" max="15" width="23.71" hidden="0" customWidth="1"/>
+    <col min="16" max="16" width="23.71" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="15.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1318,13 +1417,25 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C2" t="n">
         <v>5000</v>
@@ -1354,10 +1465,22 @@
         <v>10000</v>
       </c>
       <c r="L2" t="n">
-        <v>50000</v>
-      </c>
-      <c r="M2" t="s">
-        <v>14</v>
+        <v>6</v>
+      </c>
+      <c r="M2" t="n">
+        <v>20</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="O2" t="n">
+        <v>1800</v>
+      </c>
+      <c r="P2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="3">
@@ -1365,7 +1488,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C3" t="n">
         <v>5000</v>
@@ -1395,10 +1518,22 @@
         <v>10000</v>
       </c>
       <c r="L3" t="n">
-        <v>50000</v>
-      </c>
-      <c r="M3" t="s">
-        <v>14</v>
+        <v>6</v>
+      </c>
+      <c r="M3" t="n">
+        <v>20</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="O3" t="n">
+        <v>1800</v>
+      </c>
+      <c r="P3" t="n">
+        <v>2000</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="4">
@@ -1406,7 +1541,7 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C4" t="n">
         <v>5000</v>
@@ -1436,10 +1571,22 @@
         <v>10000</v>
       </c>
       <c r="L4" t="n">
-        <v>50000</v>
-      </c>
-      <c r="M4" t="s">
-        <v>14</v>
+        <v>6</v>
+      </c>
+      <c r="M4" t="n">
+        <v>20</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="O4" t="n">
+        <v>1800</v>
+      </c>
+      <c r="P4" t="n">
+        <v>2000</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="5">
@@ -1447,7 +1594,7 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C5" t="n">
         <v>5000</v>
@@ -1477,10 +1624,22 @@
         <v>10000</v>
       </c>
       <c r="L5" t="n">
-        <v>50000</v>
-      </c>
-      <c r="M5" t="s">
-        <v>14</v>
+        <v>6</v>
+      </c>
+      <c r="M5" t="n">
+        <v>20</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="O5" t="n">
+        <v>1800</v>
+      </c>
+      <c r="P5" t="n">
+        <v>2000</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -1514,22 +1673,23 @@
     <col min="11" max="11" width="12.71" hidden="0" customWidth="1"/>
     <col min="12" max="12" width="9.71" hidden="0" customWidth="1"/>
     <col min="13" max="13" width="9.71" hidden="0" customWidth="1"/>
-    <col min="14" max="14" width="26.71" hidden="0" customWidth="1"/>
-    <col min="15" max="15" width="28.71" hidden="0" customWidth="1"/>
-    <col min="16" max="16" width="13.71" hidden="0" customWidth="1"/>
+    <col min="14" max="14" width="22.71" hidden="0" customWidth="1"/>
+    <col min="15" max="15" width="26.71" hidden="0" customWidth="1"/>
+    <col min="16" max="16" width="28.71" hidden="0" customWidth="1"/>
     <col min="17" max="17" width="13.71" hidden="0" customWidth="1"/>
-    <col min="18" max="18" width="10.71" hidden="0" customWidth="1"/>
-    <col min="19" max="19" width="8.71" hidden="0" customWidth="1"/>
-    <col min="20" max="20" width="13.71" hidden="0" customWidth="1"/>
-    <col min="21" max="21" width="8.71" hidden="0" customWidth="1"/>
-    <col min="22" max="22" width="12.71" hidden="0" customWidth="1"/>
-    <col min="23" max="23" width="13.71" hidden="0" customWidth="1"/>
-    <col min="24" max="24" width="16.71" hidden="0" customWidth="1"/>
-    <col min="25" max="25" width="12.71" hidden="0" customWidth="1"/>
-    <col min="26" max="26" width="9.71" hidden="0" customWidth="1"/>
-    <col min="27" max="27" width="13.71" hidden="0" customWidth="1"/>
-    <col min="28" max="28" width="12.71" hidden="0" customWidth="1"/>
-    <col min="29" max="29" width="15.71" hidden="0" customWidth="1"/>
+    <col min="18" max="18" width="13.71" hidden="0" customWidth="1"/>
+    <col min="19" max="19" width="10.71" hidden="0" customWidth="1"/>
+    <col min="20" max="20" width="8.71" hidden="0" customWidth="1"/>
+    <col min="21" max="21" width="13.71" hidden="0" customWidth="1"/>
+    <col min="22" max="22" width="8.71" hidden="0" customWidth="1"/>
+    <col min="23" max="23" width="12.71" hidden="0" customWidth="1"/>
+    <col min="24" max="24" width="13.71" hidden="0" customWidth="1"/>
+    <col min="25" max="25" width="16.71" hidden="0" customWidth="1"/>
+    <col min="26" max="26" width="12.71" hidden="0" customWidth="1"/>
+    <col min="27" max="27" width="9.71" hidden="0" customWidth="1"/>
+    <col min="28" max="28" width="13.71" hidden="0" customWidth="1"/>
+    <col min="29" max="29" width="12.71" hidden="0" customWidth="1"/>
+    <col min="30" max="30" width="15.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1546,79 +1706,82 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="V1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="W1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="Y1" s="1" t="s">
-        <v>35</v>
-      </c>
       <c r="Z1" s="1" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>12</v>
+        <v>43</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="2">
@@ -1626,7 +1789,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C2" t="n">
         <v>5000</v>
@@ -1662,52 +1825,55 @@
         <v>1535</v>
       </c>
       <c r="N2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O2" t="n">
         <v>4990</v>
       </c>
-      <c r="O2" t="n">
+      <c r="P2" t="n">
         <v>99.8</v>
       </c>
-      <c r="P2" t="n">
+      <c r="Q2" t="n">
         <v>53.63</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="R2" t="n">
         <v>30.01</v>
       </c>
-      <c r="R2" t="n">
+      <c r="S2" t="n">
         <v>66.4</v>
       </c>
-      <c r="S2" t="n">
+      <c r="T2" t="n">
         <v>23.98</v>
       </c>
-      <c r="T2" t="n">
+      <c r="U2" t="n">
         <v>93</v>
       </c>
-      <c r="U2" t="n">
+      <c r="V2" t="n">
         <v>20</v>
       </c>
-      <c r="V2" t="n">
+      <c r="W2" t="n">
         <v>5000</v>
       </c>
-      <c r="W2" t="n">
+      <c r="X2" t="n">
         <v>0</v>
       </c>
-      <c r="X2" t="n">
+      <c r="Y2" t="n">
         <v>100</v>
       </c>
-      <c r="Y2" t="n">
+      <c r="Z2" t="n">
         <v>7469020</v>
       </c>
-      <c r="Z2" t="n">
+      <c r="AA2" t="n">
         <v>5000</v>
       </c>
-      <c r="AA2" t="s">
-        <v>14</v>
-      </c>
       <c r="AB2" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="AC2" t="s">
-        <v>14</v>
+        <v>18</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="3">
@@ -1715,7 +1881,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C3" t="n">
         <v>5000</v>
@@ -1751,52 +1917,55 @@
         <v>1524</v>
       </c>
       <c r="N3" t="n">
+        <v>3</v>
+      </c>
+      <c r="O3" t="n">
         <v>4991</v>
       </c>
-      <c r="O3" t="n">
+      <c r="P3" t="n">
         <v>99.82</v>
       </c>
-      <c r="P3" t="n">
+      <c r="Q3" t="n">
         <v>55.09</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="R3" t="n">
         <v>30.02</v>
       </c>
-      <c r="R3" t="n">
+      <c r="S3" t="n">
         <v>65.25</v>
       </c>
-      <c r="S3" t="n">
+      <c r="T3" t="n">
         <v>23.94</v>
       </c>
-      <c r="T3" t="n">
+      <c r="U3" t="n">
         <v>93</v>
       </c>
-      <c r="U3" t="n">
+      <c r="V3" t="n">
         <v>20</v>
       </c>
-      <c r="V3" t="n">
+      <c r="W3" t="n">
         <v>5000</v>
       </c>
-      <c r="W3" t="n">
+      <c r="X3" t="n">
         <v>0</v>
       </c>
-      <c r="X3" t="n">
+      <c r="Y3" t="n">
         <v>100</v>
       </c>
-      <c r="Y3" t="n">
+      <c r="Z3" t="n">
         <v>7440979</v>
       </c>
-      <c r="Z3" t="n">
+      <c r="AA3" t="n">
         <v>5000</v>
       </c>
-      <c r="AA3" t="s">
-        <v>14</v>
-      </c>
       <c r="AB3" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="AC3" t="s">
-        <v>14</v>
+        <v>18</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="4">
@@ -1804,7 +1973,7 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C4" t="n">
         <v>5000</v>
@@ -1840,52 +2009,55 @@
         <v>1524</v>
       </c>
       <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
         <v>4995</v>
       </c>
-      <c r="O4" t="n">
+      <c r="P4" t="n">
         <v>99.9</v>
       </c>
-      <c r="P4" t="n">
+      <c r="Q4" t="n">
         <v>54.55</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="R4" t="n">
         <v>30.03</v>
       </c>
-      <c r="R4" t="n">
+      <c r="S4" t="n">
         <v>66.86</v>
       </c>
-      <c r="S4" t="n">
+      <c r="T4" t="n">
         <v>24.17</v>
       </c>
-      <c r="T4" t="n">
+      <c r="U4" t="n">
         <v>93</v>
       </c>
-      <c r="U4" t="n">
+      <c r="V4" t="n">
         <v>20</v>
       </c>
-      <c r="V4" t="n">
+      <c r="W4" t="n">
         <v>5000</v>
       </c>
-      <c r="W4" t="n">
+      <c r="X4" t="n">
         <v>0</v>
       </c>
-      <c r="X4" t="n">
+      <c r="Y4" t="n">
         <v>100</v>
       </c>
-      <c r="Y4" t="n">
+      <c r="Z4" t="n">
         <v>7538203</v>
       </c>
-      <c r="Z4" t="n">
+      <c r="AA4" t="n">
         <v>5000</v>
       </c>
-      <c r="AA4" t="s">
-        <v>14</v>
-      </c>
       <c r="AB4" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="AC4" t="s">
-        <v>14</v>
+        <v>18</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="5">
@@ -1893,7 +2065,7 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C5" t="n">
         <v>5000</v>
@@ -1929,52 +2101,55 @@
         <v>1523</v>
       </c>
       <c r="N5" t="n">
+        <v>1</v>
+      </c>
+      <c r="O5" t="n">
         <v>4993</v>
       </c>
-      <c r="O5" t="n">
+      <c r="P5" t="n">
         <v>99.86</v>
       </c>
-      <c r="P5" t="n">
+      <c r="Q5" t="n">
         <v>54.51</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="R5" t="n">
         <v>30.02</v>
       </c>
-      <c r="R5" t="n">
+      <c r="S5" t="n">
         <v>67.67</v>
       </c>
-      <c r="S5" t="n">
+      <c r="T5" t="n">
         <v>24.17</v>
       </c>
-      <c r="T5" t="n">
+      <c r="U5" t="n">
         <v>93</v>
       </c>
-      <c r="U5" t="n">
+      <c r="V5" t="n">
         <v>20</v>
       </c>
-      <c r="V5" t="n">
+      <c r="W5" t="n">
         <v>5000</v>
       </c>
-      <c r="W5" t="n">
+      <c r="X5" t="n">
         <v>0</v>
       </c>
-      <c r="X5" t="n">
+      <c r="Y5" t="n">
         <v>100</v>
       </c>
-      <c r="Y5" t="n">
+      <c r="Z5" t="n">
         <v>7514395</v>
       </c>
-      <c r="Z5" t="n">
+      <c r="AA5" t="n">
         <v>5000</v>
       </c>
-      <c r="AA5" t="s">
-        <v>14</v>
-      </c>
       <c r="AB5" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="AC5" t="s">
-        <v>14</v>
+        <v>18</v>
+      </c>
+      <c r="AD5" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -2002,541 +2177,596 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
         <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B3" t="s">
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B4" t="s">
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B5" t="s">
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B6" t="s">
         <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B7" t="s">
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B8" t="s">
         <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B9" t="s">
         <v>7</v>
       </c>
       <c r="C9" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B10" t="s">
         <v>8</v>
       </c>
       <c r="C10" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B11" t="s">
         <v>9</v>
       </c>
       <c r="C11" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B12" t="s">
         <v>10</v>
       </c>
       <c r="C12" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B13" t="s">
         <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B14" t="s">
         <v>12</v>
       </c>
       <c r="C14" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="B15" t="s">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="C15" t="s">
-        <v>43</v>
+        <v>61</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="B16" t="s">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C16" t="s">
-        <v>44</v>
+        <v>62</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="B17" t="s">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="C17" t="s">
-        <v>45</v>
+        <v>63</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="B18" t="s">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="C18" t="s">
-        <v>46</v>
+        <v>64</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B19" t="s">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="C19" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B20" t="s">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="C20" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B21" t="s">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="C21" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B22" t="s">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="C22" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B23" t="s">
         <v>22</v>
       </c>
       <c r="C23" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B24" t="s">
         <v>23</v>
       </c>
       <c r="C24" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B25" t="s">
         <v>24</v>
       </c>
       <c r="C25" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B26" t="s">
         <v>25</v>
       </c>
       <c r="C26" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B27" t="s">
         <v>26</v>
       </c>
       <c r="C27" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B28" t="s">
         <v>27</v>
       </c>
       <c r="C28" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B29" t="s">
         <v>28</v>
       </c>
       <c r="C29" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B30" t="s">
         <v>29</v>
       </c>
       <c r="C30" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B31" t="s">
         <v>30</v>
       </c>
       <c r="C31" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B32" t="s">
         <v>31</v>
       </c>
       <c r="C32" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B33" t="s">
         <v>32</v>
       </c>
       <c r="C33" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B34" t="s">
         <v>33</v>
       </c>
       <c r="C34" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B35" t="s">
         <v>34</v>
       </c>
       <c r="C35" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B36" t="s">
-        <v>4</v>
+        <v>35</v>
       </c>
       <c r="C36" t="s">
-        <v>47</v>
+        <v>79</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B37" t="s">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="C37" t="s">
-        <v>48</v>
+        <v>80</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B38" t="s">
-        <v>6</v>
+        <v>37</v>
       </c>
       <c r="C38" t="s">
-        <v>49</v>
+        <v>81</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B39" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C39" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B40" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C40" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B41" t="s">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="C41" t="s">
-        <v>76</v>
+        <v>52</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B42" t="s">
-        <v>38</v>
+        <v>5</v>
       </c>
       <c r="C42" t="s">
-        <v>77</v>
+        <v>53</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B43" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C43" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="B44" t="s">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="C44" t="s">
-        <v>44</v>
+        <v>84</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="B45" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="C45" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="B46" t="s">
-        <v>81</v>
+        <v>42</v>
       </c>
       <c r="C46" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="B47" t="s">
-        <v>83</v>
+        <v>43</v>
       </c>
       <c r="C47" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="B48" t="s">
-        <v>85</v>
+        <v>16</v>
       </c>
       <c r="C48" t="s">
-        <v>86</v>
+        <v>64</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="B49" t="s">
-        <v>87</v>
+        <v>1</v>
       </c>
       <c r="C49" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s">
         <v>88</v>
+      </c>
+      <c r="B50" t="s">
+        <v>89</v>
+      </c>
+      <c r="C50" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="s">
+        <v>88</v>
+      </c>
+      <c r="B51" t="s">
+        <v>91</v>
+      </c>
+      <c r="C51" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s">
+        <v>88</v>
+      </c>
+      <c r="B52" t="s">
+        <v>93</v>
+      </c>
+      <c r="C52" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="s">
+        <v>88</v>
+      </c>
+      <c r="B53" t="s">
+        <v>95</v>
+      </c>
+      <c r="C53" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="s">
+        <v>88</v>
+      </c>
+      <c r="B54" t="s">
+        <v>97</v>
+      </c>
+      <c r="C54" t="s">
+        <v>98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>